<commit_message>
updated for paper figures
</commit_message>
<xml_diff>
--- a/liver TAG tracing kinetics/Chase Fasted/chase data.xlsx
+++ b/liver TAG tracing kinetics/Chase Fasted/chase data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10810"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11003"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/boyuan/Desktop/Harvard/Research/Energy Metabolism Atlas/liver TAG tracing kinetics/chase/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/boyuan/Desktop/Harvard/Research/Energy Metabolism Atlas/liver TAG tracing kinetics/Chase Fasted/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{6F8CE429-9CBF-8148-8BBF-00E1C90C6E53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2229FDC-EFBE-4E42-A2AD-691C2FE4FFC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="740" windowWidth="30240" windowHeight="18900" activeTab="3" xr2:uid="{FCC9DE73-AA74-8B43-BD8F-F00FF2F647E3}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="38400" windowHeight="21600" activeTab="7" xr2:uid="{FCC9DE73-AA74-8B43-BD8F-F00FF2F647E3}"/>
   </bookViews>
   <sheets>
     <sheet name="chase_serum_middle_point" sheetId="2" r:id="rId1"/>
@@ -329,9 +329,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="166" formatCode="0.0"/>
+    <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="22" x14ac:knownFonts="1">
+  <fonts count="21" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -471,12 +471,6 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Tahoma"/>
-      <family val="2"/>
     </font>
     <font>
       <b/>
@@ -843,7 +837,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -857,15 +851,14 @@
     </xf>
     <xf numFmtId="18" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="18" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="2" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
@@ -877,7 +870,7 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -4160,268 +4153,268 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A1" s="15" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="15" t="s">
+      <c r="A1" s="14" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="15" t="s">
+      <c r="C1" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="15" t="s">
+      <c r="D1" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="15" t="s">
+      <c r="E1" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="15" t="s">
+      <c r="F1" s="14" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="15" t="s">
+      <c r="G1" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="15" t="s">
+      <c r="H1" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="15" t="s">
+      <c r="I1" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="15" t="s">
+      <c r="J1" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="15" t="s">
+      <c r="K1" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="15" t="s">
+      <c r="L1" s="14" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A2" s="15" t="s">
+      <c r="A2" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="B2" s="15" t="s">
+      <c r="B2" s="14" t="s">
         <v>33</v>
       </c>
-      <c r="C2" s="15" t="s">
+      <c r="C2" s="14" t="s">
         <v>34</v>
       </c>
-      <c r="D2" s="15">
+      <c r="D2" s="14">
         <v>9382123</v>
       </c>
-      <c r="E2" s="15">
+      <c r="E2" s="14">
         <v>8189636.5</v>
       </c>
-      <c r="F2" s="15">
+      <c r="F2" s="14">
         <v>13830656</v>
       </c>
-      <c r="G2" s="15">
+      <c r="G2" s="14">
         <v>17404450</v>
       </c>
-      <c r="H2" s="15">
+      <c r="H2" s="14">
         <v>12048172</v>
       </c>
-      <c r="I2" s="15">
+      <c r="I2" s="14">
         <v>24840882</v>
       </c>
-      <c r="J2" s="15">
+      <c r="J2" s="14">
         <v>21390064</v>
       </c>
-      <c r="K2" s="15">
+      <c r="K2" s="14">
         <v>13743153</v>
       </c>
-      <c r="L2" s="15">
+      <c r="L2" s="14">
         <v>10305718</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A3" s="15" t="s">
+      <c r="A3" s="14" t="s">
         <v>35</v>
       </c>
-      <c r="B3" s="15" t="s">
+      <c r="B3" s="14" t="s">
         <v>33</v>
       </c>
-      <c r="C3" s="15" t="s">
+      <c r="C3" s="14" t="s">
         <v>34</v>
       </c>
-      <c r="D3" s="15">
+      <c r="D3" s="14">
         <v>1645781.62</v>
       </c>
-      <c r="E3" s="15">
+      <c r="E3" s="14">
         <v>1466826.38</v>
       </c>
-      <c r="F3" s="15">
+      <c r="F3" s="14">
         <v>2465863.25</v>
       </c>
-      <c r="G3" s="15">
+      <c r="G3" s="14">
         <v>3191001.25</v>
       </c>
-      <c r="H3" s="15">
+      <c r="H3" s="14">
         <v>2193899.25</v>
       </c>
-      <c r="I3" s="15">
+      <c r="I3" s="14">
         <v>4631714.5</v>
       </c>
-      <c r="J3" s="15">
+      <c r="J3" s="14">
         <v>4013439.75</v>
       </c>
-      <c r="K3" s="15">
+      <c r="K3" s="14">
         <v>2462002</v>
       </c>
-      <c r="L3" s="15">
+      <c r="L3" s="14">
         <v>1734284.38</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A4" s="15" t="s">
+      <c r="A4" s="14" t="s">
         <v>36</v>
       </c>
-      <c r="B4" s="15" t="s">
+      <c r="B4" s="14" t="s">
         <v>33</v>
       </c>
-      <c r="C4" s="15" t="s">
+      <c r="C4" s="14" t="s">
         <v>34</v>
       </c>
-      <c r="D4" s="15">
+      <c r="D4" s="14">
         <v>9847.85</v>
       </c>
-      <c r="E4" s="15">
-        <v>0</v>
-      </c>
-      <c r="F4" s="15">
-        <v>0</v>
-      </c>
-      <c r="G4" s="15">
+      <c r="E4" s="14">
+        <v>0</v>
+      </c>
+      <c r="F4" s="14">
+        <v>0</v>
+      </c>
+      <c r="G4" s="14">
         <v>46521.75</v>
       </c>
-      <c r="H4" s="15">
+      <c r="H4" s="14">
         <v>3492.97</v>
       </c>
-      <c r="I4" s="15">
+      <c r="I4" s="14">
         <v>13774.23</v>
       </c>
-      <c r="J4" s="15">
+      <c r="J4" s="14">
         <v>39531.769999999997</v>
       </c>
-      <c r="K4" s="15">
-        <v>0</v>
-      </c>
-      <c r="L4" s="15">
+      <c r="K4" s="14">
+        <v>0</v>
+      </c>
+      <c r="L4" s="14">
         <v>6730.54</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A5" s="15" t="s">
+      <c r="A5" s="14" t="s">
         <v>37</v>
       </c>
-      <c r="B5" s="15" t="s">
+      <c r="B5" s="14" t="s">
         <v>33</v>
       </c>
-      <c r="C5" s="15" t="s">
+      <c r="C5" s="14" t="s">
         <v>34</v>
       </c>
-      <c r="D5" s="15">
+      <c r="D5" s="14">
         <v>11185.35</v>
       </c>
-      <c r="E5" s="15">
+      <c r="E5" s="14">
         <v>28494.48</v>
       </c>
-      <c r="F5" s="15">
+      <c r="F5" s="14">
         <v>33522.120000000003</v>
       </c>
-      <c r="G5" s="15">
+      <c r="G5" s="14">
         <v>136620.81</v>
       </c>
-      <c r="H5" s="15">
+      <c r="H5" s="14">
         <v>39372.44</v>
       </c>
-      <c r="I5" s="15">
+      <c r="I5" s="14">
         <v>86553.07</v>
       </c>
-      <c r="J5" s="15">
+      <c r="J5" s="14">
         <v>129231.84</v>
       </c>
-      <c r="K5" s="15">
+      <c r="K5" s="14">
         <v>33239.83</v>
       </c>
-      <c r="L5" s="15">
+      <c r="L5" s="14">
         <v>20854.689999999999</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A6" s="15" t="s">
+      <c r="A6" s="14" t="s">
         <v>38</v>
       </c>
-      <c r="B6" s="15" t="s">
+      <c r="B6" s="14" t="s">
         <v>33</v>
       </c>
-      <c r="C6" s="15" t="s">
+      <c r="C6" s="14" t="s">
         <v>34</v>
       </c>
-      <c r="D6" s="15">
+      <c r="D6" s="14">
         <v>416481.03</v>
       </c>
-      <c r="E6" s="15">
+      <c r="E6" s="14">
         <v>318136.88</v>
       </c>
-      <c r="F6" s="15">
+      <c r="F6" s="14">
         <v>589941.5</v>
       </c>
-      <c r="G6" s="15">
+      <c r="G6" s="14">
         <v>2106212.25</v>
       </c>
-      <c r="H6" s="15">
+      <c r="H6" s="14">
         <v>641473.06000000006</v>
       </c>
-      <c r="I6" s="15">
+      <c r="I6" s="14">
         <v>1287164.1200000001</v>
       </c>
-      <c r="J6" s="15">
+      <c r="J6" s="14">
         <v>3465542.25</v>
       </c>
-      <c r="K6" s="15">
+      <c r="K6" s="14">
         <v>559322.31000000006</v>
       </c>
-      <c r="L6" s="15">
+      <c r="L6" s="14">
         <v>555968.25</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A7" s="15" t="s">
+      <c r="A7" s="14" t="s">
         <v>41</v>
       </c>
-      <c r="B7" s="15" t="s">
+      <c r="B7" s="14" t="s">
         <v>33</v>
       </c>
-      <c r="C7" s="15" t="s">
+      <c r="C7" s="14" t="s">
         <v>34</v>
       </c>
-      <c r="D7" s="15">
+      <c r="D7" s="14">
         <v>119743.29</v>
       </c>
-      <c r="E7" s="15">
+      <c r="E7" s="14">
         <v>10096.11</v>
       </c>
-      <c r="F7" s="15">
+      <c r="F7" s="14">
         <v>34831.4</v>
       </c>
-      <c r="G7" s="15">
-        <v>0</v>
-      </c>
-      <c r="H7" s="15">
-        <v>0</v>
-      </c>
-      <c r="I7" s="15">
+      <c r="G7" s="14">
+        <v>0</v>
+      </c>
+      <c r="H7" s="14">
+        <v>0</v>
+      </c>
+      <c r="I7" s="14">
         <v>56898.33</v>
       </c>
-      <c r="J7" s="15">
+      <c r="J7" s="14">
         <v>166160.89000000001</v>
       </c>
-      <c r="K7" s="15">
+      <c r="K7" s="14">
         <v>79630.66</v>
       </c>
-      <c r="L7" s="15">
+      <c r="L7" s="14">
         <v>16623.32</v>
       </c>
     </row>
@@ -4684,20 +4677,19 @@
     <col min="1" max="1" width="16.5" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="11.6640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11.6640625" style="6" bestFit="1" customWidth="1"/>
-    <col min="5" max="16384" width="10.83203125" style="9"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="B1" s="10" t="s">
+      <c r="B1" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="C1" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="D1" s="11" t="s">
+      <c r="D1" s="10" t="s">
         <v>75</v>
       </c>
     </row>
@@ -4711,7 +4703,7 @@
       <c r="C2" s="4">
         <v>0.71527777777777779</v>
       </c>
-      <c r="D2" s="12">
+      <c r="D2" s="11">
         <f>(C2-B2)*24</f>
         <v>0.50000000000000089</v>
       </c>
@@ -4726,7 +4718,7 @@
       <c r="C3" s="4">
         <v>0.71736111111111112</v>
       </c>
-      <c r="D3" s="12">
+      <c r="D3" s="11">
         <f>(C3-B3)*24</f>
         <v>0.5166666666666675</v>
       </c>
@@ -4741,13 +4733,13 @@
       <c r="C4" s="4">
         <v>0.72083333333333333</v>
       </c>
-      <c r="D4" s="12">
+      <c r="D4" s="11">
         <f>(C4-B4)*24</f>
         <v>0.31666666666666554</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="13" t="s">
+      <c r="A5" s="12" t="s">
         <v>22</v>
       </c>
       <c r="B5" s="8">
@@ -4756,7 +4748,7 @@
       <c r="C5" s="8">
         <v>0.72013888888888888</v>
       </c>
-      <c r="D5" s="14">
+      <c r="D5" s="13">
         <f>(C5-B5)*24</f>
         <v>0.24999999999999911</v>
       </c>
@@ -4771,7 +4763,7 @@
       <c r="C6" s="4">
         <v>0.77777777777777779</v>
       </c>
-      <c r="D6" s="12">
+      <c r="D6" s="11">
         <f t="shared" ref="D6:D32" si="0">(C6-B6)*24</f>
         <v>2.0000000000000009</v>
       </c>
@@ -4786,7 +4778,7 @@
       <c r="C7" s="4">
         <v>0.78263888888888888</v>
       </c>
-      <c r="D7" s="12">
+      <c r="D7" s="11">
         <f t="shared" si="0"/>
         <v>2.0833333333333339</v>
       </c>
@@ -4801,7 +4793,7 @@
       <c r="C8" s="4">
         <v>0.78680555555555554</v>
       </c>
-      <c r="D8" s="12">
+      <c r="D8" s="11">
         <f t="shared" si="0"/>
         <v>2.1333333333333337</v>
       </c>
@@ -4816,7 +4808,7 @@
       <c r="C9" s="4">
         <v>0.7</v>
       </c>
-      <c r="D9" s="12">
+      <c r="D9" s="11">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -4831,7 +4823,7 @@
       <c r="C10" s="4">
         <v>0.76736111111111116</v>
       </c>
-      <c r="D10" s="12">
+      <c r="D10" s="11">
         <f t="shared" si="0"/>
         <v>1.5666666666666691</v>
       </c>
@@ -4846,7 +4838,7 @@
       <c r="C11" s="4">
         <v>0.74861111111111112</v>
       </c>
-      <c r="D11" s="12">
+      <c r="D11" s="11">
         <f t="shared" si="0"/>
         <v>1.0666666666666655</v>
       </c>
@@ -4861,7 +4853,7 @@
       <c r="C12" s="4">
         <v>0.70625000000000004</v>
       </c>
-      <c r="D12" s="12">
+      <c r="D12" s="11">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -4876,13 +4868,13 @@
       <c r="C13" s="4">
         <v>0.75486111111111109</v>
       </c>
-      <c r="D13" s="12">
+      <c r="D13" s="11">
         <f t="shared" si="0"/>
         <v>1.133333333333332</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="13" t="s">
+      <c r="A14" s="12" t="s">
         <v>31</v>
       </c>
       <c r="B14" s="8">
@@ -4891,7 +4883,7 @@
       <c r="C14" s="8">
         <v>0.76041666666666663</v>
       </c>
-      <c r="D14" s="14">
+      <c r="D14" s="13">
         <f t="shared" si="0"/>
         <v>1.216666666666665</v>
       </c>
@@ -4906,7 +4898,7 @@
       <c r="C15" s="4">
         <v>0.77777777777777779</v>
       </c>
-      <c r="D15" s="12">
+      <c r="D15" s="11">
         <f t="shared" si="0"/>
         <v>2.0000000000000009</v>
       </c>
@@ -4921,7 +4913,7 @@
       <c r="C16" s="4">
         <v>0.78263888888888888</v>
       </c>
-      <c r="D16" s="12">
+      <c r="D16" s="11">
         <f t="shared" si="0"/>
         <v>2.0833333333333339</v>
       </c>
@@ -4936,7 +4928,7 @@
       <c r="C17" s="4">
         <v>0.78680555555555554</v>
       </c>
-      <c r="D17" s="12">
+      <c r="D17" s="11">
         <f t="shared" si="0"/>
         <v>2.1333333333333337</v>
       </c>
@@ -4951,7 +4943,7 @@
       <c r="C18" s="4">
         <v>0.7</v>
       </c>
-      <c r="D18" s="12">
+      <c r="D18" s="11">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -4966,7 +4958,7 @@
       <c r="C19" s="4">
         <v>0.76736111111111116</v>
       </c>
-      <c r="D19" s="12">
+      <c r="D19" s="11">
         <f t="shared" si="0"/>
         <v>1.5666666666666691</v>
       </c>
@@ -4981,7 +4973,7 @@
       <c r="C20" s="4">
         <v>0.74861111111111112</v>
       </c>
-      <c r="D20" s="12">
+      <c r="D20" s="11">
         <f t="shared" si="0"/>
         <v>1.0666666666666655</v>
       </c>
@@ -4996,7 +4988,7 @@
       <c r="C21" s="4">
         <v>0.70625000000000004</v>
       </c>
-      <c r="D21" s="12">
+      <c r="D21" s="11">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -5011,13 +5003,13 @@
       <c r="C22" s="4">
         <v>0.75486111111111109</v>
       </c>
-      <c r="D22" s="12">
+      <c r="D22" s="11">
         <f t="shared" si="0"/>
         <v>1.133333333333332</v>
       </c>
     </row>
     <row r="23" spans="1:4" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="13" t="s">
+      <c r="A23" s="12" t="s">
         <v>11</v>
       </c>
       <c r="B23" s="8">
@@ -5026,7 +5018,7 @@
       <c r="C23" s="8">
         <v>0.76041666666666663</v>
       </c>
-      <c r="D23" s="14">
+      <c r="D23" s="13">
         <f t="shared" si="0"/>
         <v>1.216666666666665</v>
       </c>
@@ -5041,7 +5033,7 @@
       <c r="C24" s="4">
         <v>0.77777777777777779</v>
       </c>
-      <c r="D24" s="12">
+      <c r="D24" s="11">
         <f t="shared" si="0"/>
         <v>2.0000000000000009</v>
       </c>
@@ -5056,7 +5048,7 @@
       <c r="C25" s="4">
         <v>0.78263888888888888</v>
       </c>
-      <c r="D25" s="12">
+      <c r="D25" s="11">
         <f t="shared" si="0"/>
         <v>2.0833333333333339</v>
       </c>
@@ -5071,7 +5063,7 @@
       <c r="C26" s="4">
         <v>0.78680555555555554</v>
       </c>
-      <c r="D26" s="12">
+      <c r="D26" s="11">
         <f t="shared" si="0"/>
         <v>2.1333333333333337</v>
       </c>
@@ -5086,7 +5078,7 @@
       <c r="C27" s="4">
         <v>0.7</v>
       </c>
-      <c r="D27" s="12">
+      <c r="D27" s="11">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -5101,7 +5093,7 @@
       <c r="C28" s="4">
         <v>0.76736111111111116</v>
       </c>
-      <c r="D28" s="12">
+      <c r="D28" s="11">
         <f t="shared" si="0"/>
         <v>1.5666666666666691</v>
       </c>
@@ -5116,7 +5108,7 @@
       <c r="C29" s="4">
         <v>0.74861111111111112</v>
       </c>
-      <c r="D29" s="12">
+      <c r="D29" s="11">
         <f t="shared" si="0"/>
         <v>1.0666666666666655</v>
       </c>
@@ -5131,7 +5123,7 @@
       <c r="C30" s="4">
         <v>0.70625000000000004</v>
       </c>
-      <c r="D30" s="12">
+      <c r="D30" s="11">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -5146,7 +5138,7 @@
       <c r="C31" s="4">
         <v>0.75486111111111109</v>
       </c>
-      <c r="D31" s="12">
+      <c r="D31" s="11">
         <f t="shared" si="0"/>
         <v>1.133333333333332</v>
       </c>
@@ -5161,7 +5153,7 @@
       <c r="C32" s="4">
         <v>0.76041666666666663</v>
       </c>
-      <c r="D32" s="12">
+      <c r="D32" s="11">
         <f t="shared" si="0"/>
         <v>1.216666666666665</v>
       </c>

</xml_diff>